<commit_message>
Pre-deploy scrub: redact named contacts in market maps, gitignore Claude cache, restore legacy note on player_overrides.xlsx
- Replaced 140 named contacts in Validated By columns across BEL/ENG/FRA/DEU/NLD market maps with [redacted]
- Cleaned authoring-draft phrasing in manual_flags.xlsx notes_source column
- Updated CLAUDE.md project header wordmark to RMC
- Redacted personal email in BACKLOG.md
- Added .claude/ to .gitignore, removed tracked settings.local.json
- Restored legacy/superseded note on data/player_overrides.xlsx in CLAUDE.md

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/manual_flags.xlsx
+++ b/data/manual_flags.xlsx
@@ -19823,7 +19823,7 @@
       </c>
       <c r="P294" s="5" t="inlineStr">
         <is>
-          <t>Ryan flag (Day 5): FFP / financial pressure — public must-sell</t>
+          <t>Manual flag: FFP / financial pressure — public must-sell</t>
         </is>
       </c>
       <c r="Q294" s="2" t="inlineStr"/>
@@ -20603,7 +20603,7 @@
       </c>
       <c r="P306" s="5" t="inlineStr">
         <is>
-          <t>Ryan flag (Day 5): FFP / financial pressure — public must-sell</t>
+          <t>Manual flag: FFP / financial pressure — public must-sell</t>
         </is>
       </c>
       <c r="Q306" s="2" t="inlineStr"/>

</xml_diff>